<commit_message>
Implement premium ticket design replica from image
</commit_message>
<xml_diff>
--- a/Data_Pendaftaran_Event.xlsx
+++ b/Data_Pendaftaran_Event.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\E-Tiket\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92695161-FB77-476E-9931-F4A70DC3E173}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42C78845-B751-4C08-93D6-34855F2FBC91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="76">
   <si>
     <t>Nama Lengkap</t>
   </si>
@@ -246,6 +246,9 @@
   </si>
   <si>
     <t>ikhsanloris@gmail.com</t>
+  </si>
+  <si>
+    <t>Wa Lina</t>
   </si>
 </sst>
 </file>
@@ -724,9 +727,9 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>24</v>
+        <v>75</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>25</v>
@@ -741,7 +744,7 @@
         <v>27</v>
       </c>
       <c r="F3" s="3">
-        <v>81234567802</v>
+        <v>85299383426</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>28</v>
@@ -1110,7 +1113,7 @@
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" xr:uid="{0939B43E-12EC-4E4E-87A0-60D35F24525D}"/>
-    <hyperlink ref="B3" r:id="rId2" display="mailto:sitirahma@gmail.com" xr:uid="{8E823B73-1F57-44A2-A603-4BD5F8460807}"/>
+    <hyperlink ref="B3" r:id="rId2" xr:uid="{8E823B73-1F57-44A2-A603-4BD5F8460807}"/>
     <hyperlink ref="B4" r:id="rId3" display="mailto:budisantoso@gmail.com" xr:uid="{9842F513-0339-45FE-848F-597B2EE2625B}"/>
     <hyperlink ref="B5" r:id="rId4" display="mailto:dewilestari@gmail.com" xr:uid="{9B981876-8CB5-4FDE-B2AF-4FA0C48266F2}"/>
     <hyperlink ref="B6" r:id="rId5" display="mailto:rizkymaulana@gmail.com" xr:uid="{BD7CB548-41CB-4A09-B9D2-B601E452AC9E}"/>

</xml_diff>